<commit_message>
better gitignore + violations on artificial datasets
</commit_message>
<xml_diff>
--- a/generated-output/report.xlsx
+++ b/generated-output/report.xlsx
@@ -1363,11 +1363,620 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr"/>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>qse-0.0</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>qse-0.5</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>qse-0.9</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>qse-1.0</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>shexer-unsound-0</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>shexer-sound-0</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>shexer-unsound-0.5</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>shexer-sound-0.5</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>shexer-unsound-0.9</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>shexer-sound-0.9</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>shexer-unsound-1</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>shexer-sound-1</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>play</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>voicl</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>people</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0 / 20</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>people-all</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2 / 3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0 / 19</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>15 / 15</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2 / 3</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>people-datetime</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0 / 20</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>people-schema</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0 / 20</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>10 / 10</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1 / 2</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1 / 2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>people-string</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0 / 20</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>0 / 10</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>people-two-birthday</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0 / 21</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>people-without-birthday</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0 / 19</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1 / 1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0 / 9</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>